<commit_message>
remove xlsx and keep csv
</commit_message>
<xml_diff>
--- a/Data/Rawdata/csvs/84_Hernandez_Castellano_2025.xlsx
+++ b/Data/Rawdata/csvs/84_Hernandez_Castellano_2025.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Dropbox\Spanish_Bees\done\Data_MJ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\OneDrive\Escritorio\Maria_Jose\Proyectos_git\IberianBees\Data\Rawdata\csvs\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -15,7 +15,7 @@
     <sheet name="Template" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template!$A$1:$AA$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Template!$A$1:$AA$110</definedName>
   </definedNames>
   <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2072" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2090" uniqueCount="198">
   <si>
     <t>Genus</t>
   </si>
@@ -622,6 +622,12 @@
   </si>
   <si>
     <t>10.2436/20.1502.01.222</t>
+  </si>
+  <si>
+    <t>incertae</t>
+  </si>
+  <si>
+    <t>sedis</t>
   </si>
 </sst>
 </file>
@@ -1002,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AA109"/>
+  <dimension ref="A1:AA110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.33203125" customWidth="1"/>
@@ -1111,10 +1117,10 @@
         <v>28</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>196</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
+        <v>197</v>
       </c>
       <c r="E2" t="s">
         <v>29</v>
@@ -1179,10 +1185,10 @@
         <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D3" t="s">
         <v>28</v>
@@ -1247,13 +1253,13 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
         <v>28</v>
@@ -1324,7 +1330,7 @@
         <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
         <v>28</v>
@@ -1389,13 +1395,13 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
@@ -1460,13 +1466,13 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D7" t="s">
         <v>28</v>
@@ -1537,7 +1543,7 @@
         <v>41</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
         <v>28</v>
@@ -1605,10 +1611,10 @@
         <v>41</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
@@ -1673,13 +1679,13 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D10" t="s">
         <v>28</v>
@@ -1744,13 +1750,13 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D11" t="s">
         <v>28</v>
@@ -1818,10 +1824,10 @@
         <v>48</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D12" t="s">
         <v>28</v>
@@ -1886,13 +1892,13 @@
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
         <v>28</v>
@@ -1960,10 +1966,10 @@
         <v>52</v>
       </c>
       <c r="B14" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
         <v>28</v>
@@ -2031,10 +2037,10 @@
         <v>52</v>
       </c>
       <c r="B15" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
         <v>28</v>
@@ -2105,7 +2111,7 @@
         <v>56</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
         <v>28</v>
@@ -2176,7 +2182,7 @@
         <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
         <v>28</v>
@@ -2247,7 +2253,7 @@
         <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
         <v>28</v>
@@ -2318,7 +2324,7 @@
         <v>56</v>
       </c>
       <c r="C19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
         <v>28</v>
@@ -2389,7 +2395,7 @@
         <v>56</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D20" t="s">
         <v>28</v>
@@ -2460,7 +2466,7 @@
         <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
         <v>28</v>
@@ -2531,7 +2537,7 @@
         <v>56</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D22" t="s">
         <v>28</v>
@@ -2602,7 +2608,7 @@
         <v>56</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D23" t="s">
         <v>28</v>
@@ -2667,13 +2673,13 @@
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D24" t="s">
         <v>28</v>
@@ -2738,13 +2744,13 @@
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
         <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D25" t="s">
         <v>28</v>
@@ -2815,7 +2821,7 @@
         <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D26" t="s">
         <v>28</v>
@@ -2880,13 +2886,13 @@
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B27" t="s">
         <v>28</v>
       </c>
       <c r="C27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D27" t="s">
         <v>28</v>
@@ -2957,7 +2963,7 @@
         <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D28" t="s">
         <v>28</v>
@@ -3022,13 +3028,13 @@
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="C29" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D29" t="s">
         <v>28</v>
@@ -3096,10 +3102,10 @@
         <v>74</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D30" t="s">
         <v>28</v>
@@ -3164,13 +3170,13 @@
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B31" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D31" t="s">
         <v>28</v>
@@ -3241,7 +3247,7 @@
         <v>28</v>
       </c>
       <c r="C32" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D32" t="s">
         <v>28</v>
@@ -3306,13 +3312,13 @@
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B33" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="C33" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D33" t="s">
         <v>28</v>
@@ -3383,7 +3389,7 @@
         <v>82</v>
       </c>
       <c r="C34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D34" t="s">
         <v>28</v>
@@ -3454,7 +3460,7 @@
         <v>82</v>
       </c>
       <c r="C35" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D35" t="s">
         <v>28</v>
@@ -3522,10 +3528,10 @@
         <v>81</v>
       </c>
       <c r="B36" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D36" t="s">
         <v>28</v>
@@ -3596,7 +3602,7 @@
         <v>81</v>
       </c>
       <c r="C37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D37" t="s">
         <v>28</v>
@@ -3667,7 +3673,7 @@
         <v>81</v>
       </c>
       <c r="C38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D38" t="s">
         <v>28</v>
@@ -3738,7 +3744,7 @@
         <v>81</v>
       </c>
       <c r="C39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D39" t="s">
         <v>28</v>
@@ -3806,10 +3812,10 @@
         <v>81</v>
       </c>
       <c r="B40" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C40" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D40" t="s">
         <v>28</v>
@@ -3877,10 +3883,10 @@
         <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C41" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D41" t="s">
         <v>28</v>
@@ -3951,7 +3957,7 @@
         <v>92</v>
       </c>
       <c r="C42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D42" t="s">
         <v>28</v>
@@ -4022,7 +4028,7 @@
         <v>92</v>
       </c>
       <c r="C43" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D43" t="s">
         <v>28</v>
@@ -4090,10 +4096,10 @@
         <v>81</v>
       </c>
       <c r="B44" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C44" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D44" t="s">
         <v>28</v>
@@ -4164,7 +4170,7 @@
         <v>96</v>
       </c>
       <c r="C45" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D45" t="s">
         <v>28</v>
@@ -4235,7 +4241,7 @@
         <v>96</v>
       </c>
       <c r="C46" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D46" t="s">
         <v>28</v>
@@ -4306,7 +4312,7 @@
         <v>96</v>
       </c>
       <c r="C47" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D47" t="s">
         <v>28</v>
@@ -4374,10 +4380,10 @@
         <v>81</v>
       </c>
       <c r="B48" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C48" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D48" t="s">
         <v>28</v>
@@ -4448,7 +4454,7 @@
         <v>101</v>
       </c>
       <c r="C49" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D49" t="s">
         <v>28</v>
@@ -4513,13 +4519,13 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="B50" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C50" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D50" t="s">
         <v>28</v>
@@ -4590,7 +4596,7 @@
         <v>105</v>
       </c>
       <c r="C51" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D51" t="s">
         <v>28</v>
@@ -4661,7 +4667,7 @@
         <v>105</v>
       </c>
       <c r="C52" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D52" t="s">
         <v>28</v>
@@ -4729,10 +4735,10 @@
         <v>104</v>
       </c>
       <c r="B53" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C53" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D53" t="s">
         <v>28</v>
@@ -4797,13 +4803,13 @@
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B54" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C54" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D54" t="s">
         <v>28</v>
@@ -4874,7 +4880,7 @@
         <v>112</v>
       </c>
       <c r="C55" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D55" t="s">
         <v>28</v>
@@ -4945,7 +4951,7 @@
         <v>112</v>
       </c>
       <c r="C56" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D56" t="s">
         <v>28</v>
@@ -5016,7 +5022,7 @@
         <v>112</v>
       </c>
       <c r="C57" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D57" t="s">
         <v>28</v>
@@ -5087,7 +5093,7 @@
         <v>112</v>
       </c>
       <c r="C58" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D58" t="s">
         <v>28</v>
@@ -5158,7 +5164,7 @@
         <v>112</v>
       </c>
       <c r="C59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D59" t="s">
         <v>28</v>
@@ -5229,7 +5235,7 @@
         <v>112</v>
       </c>
       <c r="C60" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D60" t="s">
         <v>28</v>
@@ -5300,7 +5306,7 @@
         <v>112</v>
       </c>
       <c r="C61" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D61" t="s">
         <v>28</v>
@@ -5371,7 +5377,7 @@
         <v>112</v>
       </c>
       <c r="C62" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D62" t="s">
         <v>28</v>
@@ -5429,12 +5435,6 @@
       </c>
       <c r="V62" t="s">
         <v>195</v>
-      </c>
-      <c r="W62" t="s">
-        <v>28</v>
-      </c>
-      <c r="X62" t="s">
-        <v>28</v>
       </c>
       <c r="Y62" t="s">
         <v>194</v>
@@ -5448,7 +5448,7 @@
         <v>112</v>
       </c>
       <c r="C63" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D63" t="s">
         <v>28</v>
@@ -5525,7 +5525,7 @@
         <v>112</v>
       </c>
       <c r="C64" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D64" t="s">
         <v>28</v>
@@ -5602,7 +5602,7 @@
         <v>112</v>
       </c>
       <c r="C65" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D65" t="s">
         <v>28</v>
@@ -5679,7 +5679,7 @@
         <v>112</v>
       </c>
       <c r="C66" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D66" t="s">
         <v>28</v>
@@ -5756,7 +5756,7 @@
         <v>112</v>
       </c>
       <c r="C67" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D67" t="s">
         <v>28</v>
@@ -5833,7 +5833,7 @@
         <v>112</v>
       </c>
       <c r="C68" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D68" t="s">
         <v>28</v>
@@ -5907,10 +5907,10 @@
         <v>111</v>
       </c>
       <c r="B69" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C69" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D69" t="s">
         <v>28</v>
@@ -5984,152 +5984,152 @@
         <v>111</v>
       </c>
       <c r="B70" t="s">
+        <v>111</v>
+      </c>
+      <c r="C70" t="s">
+        <v>128</v>
+      </c>
+      <c r="D70" t="s">
+        <v>28</v>
+      </c>
+      <c r="E70" t="s">
+        <v>29</v>
+      </c>
+      <c r="F70" t="s">
+        <v>31</v>
+      </c>
+      <c r="G70" t="s">
+        <v>32</v>
+      </c>
+      <c r="H70">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I70">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J70" t="s">
+        <v>28</v>
+      </c>
+      <c r="K70">
+        <v>2024</v>
+      </c>
+      <c r="L70" t="s">
+        <v>33</v>
+      </c>
+      <c r="M70" t="s">
+        <v>28</v>
+      </c>
+      <c r="N70">
+        <v>13</v>
+      </c>
+      <c r="O70">
+        <v>19</v>
+      </c>
+      <c r="P70" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>28</v>
+      </c>
+      <c r="R70" t="s">
+        <v>28</v>
+      </c>
+      <c r="S70" t="s">
+        <v>28</v>
+      </c>
+      <c r="T70" t="s">
+        <v>28</v>
+      </c>
+      <c r="U70" t="s">
+        <v>28</v>
+      </c>
+      <c r="V70" t="s">
+        <v>195</v>
+      </c>
+      <c r="W70" t="s">
+        <v>28</v>
+      </c>
+      <c r="X70" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y70" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="71" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>111</v>
+      </c>
+      <c r="B71" t="s">
         <v>129</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C71" t="s">
         <v>130</v>
       </c>
-      <c r="D70" t="s">
-        <v>28</v>
-      </c>
-      <c r="E70" t="s">
-        <v>29</v>
-      </c>
-      <c r="F70" t="s">
-        <v>31</v>
-      </c>
-      <c r="G70" t="s">
-        <v>32</v>
-      </c>
-      <c r="H70">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I70">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J70" t="s">
-        <v>28</v>
-      </c>
-      <c r="K70">
-        <v>2024</v>
-      </c>
-      <c r="L70" t="s">
-        <v>33</v>
-      </c>
-      <c r="M70" t="s">
-        <v>28</v>
-      </c>
-      <c r="N70">
-        <v>13</v>
-      </c>
-      <c r="O70">
-        <v>19</v>
-      </c>
-      <c r="P70" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q70" t="s">
-        <v>28</v>
-      </c>
-      <c r="R70" t="s">
-        <v>28</v>
-      </c>
-      <c r="S70" t="s">
-        <v>28</v>
-      </c>
-      <c r="T70" t="s">
-        <v>28</v>
-      </c>
-      <c r="U70" t="s">
-        <v>28</v>
-      </c>
-      <c r="V70" t="s">
-        <v>195</v>
-      </c>
-      <c r="W70" t="s">
-        <v>28</v>
-      </c>
-      <c r="X70" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y70" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="71" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B71" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C71" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="D71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G71" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H71" s="4">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I71" s="4">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K71" s="4">
-        <v>2024</v>
-      </c>
-      <c r="L71" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N71" s="4">
-        <v>13</v>
-      </c>
-      <c r="O71" s="4">
-        <v>19</v>
-      </c>
-      <c r="P71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="R71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="S71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="T71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="U71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="V71" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="W71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="X71" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y71" s="4" t="s">
+      <c r="D71" t="s">
+        <v>28</v>
+      </c>
+      <c r="E71" t="s">
+        <v>29</v>
+      </c>
+      <c r="F71" t="s">
+        <v>31</v>
+      </c>
+      <c r="G71" t="s">
+        <v>32</v>
+      </c>
+      <c r="H71">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I71">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J71" t="s">
+        <v>28</v>
+      </c>
+      <c r="K71">
+        <v>2024</v>
+      </c>
+      <c r="L71" t="s">
+        <v>33</v>
+      </c>
+      <c r="M71" t="s">
+        <v>28</v>
+      </c>
+      <c r="N71">
+        <v>13</v>
+      </c>
+      <c r="O71">
+        <v>19</v>
+      </c>
+      <c r="P71" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>28</v>
+      </c>
+      <c r="R71" t="s">
+        <v>28</v>
+      </c>
+      <c r="S71" t="s">
+        <v>28</v>
+      </c>
+      <c r="T71" t="s">
+        <v>28</v>
+      </c>
+      <c r="U71" t="s">
+        <v>28</v>
+      </c>
+      <c r="V71" t="s">
+        <v>195</v>
+      </c>
+      <c r="W71" t="s">
+        <v>28</v>
+      </c>
+      <c r="X71" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y71" t="s">
         <v>194</v>
       </c>
     </row>
@@ -6141,149 +6141,149 @@
         <v>129</v>
       </c>
       <c r="C72" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H72" s="4">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I72" s="4">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K72" s="4">
+        <v>2024</v>
+      </c>
+      <c r="L72" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N72" s="4">
+        <v>13</v>
+      </c>
+      <c r="O72" s="4">
+        <v>19</v>
+      </c>
+      <c r="P72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="R72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="S72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="T72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="U72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="V72" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="W72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="X72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y72" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="73" spans="1:25" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C73" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="D72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E72" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F72" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G72" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H72" s="4">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I72" s="4">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K72" s="4">
-        <v>2024</v>
-      </c>
-      <c r="L72" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N72" s="4">
-        <v>13</v>
-      </c>
-      <c r="O72" s="4">
-        <v>19</v>
-      </c>
-      <c r="P72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="R72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="S72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="T72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="U72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="V72" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="W72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="X72" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y72" s="4" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="73" spans="1:25" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>111</v>
-      </c>
-      <c r="B73" t="s">
-        <v>129</v>
-      </c>
-      <c r="C73" t="s">
-        <v>133</v>
-      </c>
-      <c r="D73" t="s">
-        <v>28</v>
-      </c>
-      <c r="E73" t="s">
-        <v>29</v>
-      </c>
-      <c r="F73" t="s">
-        <v>31</v>
-      </c>
-      <c r="G73" t="s">
-        <v>32</v>
-      </c>
-      <c r="H73">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I73">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J73" t="s">
-        <v>28</v>
-      </c>
-      <c r="K73">
-        <v>2024</v>
-      </c>
-      <c r="L73" t="s">
-        <v>33</v>
-      </c>
-      <c r="M73" t="s">
-        <v>28</v>
-      </c>
-      <c r="N73">
-        <v>13</v>
-      </c>
-      <c r="O73">
-        <v>19</v>
-      </c>
-      <c r="P73" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q73" t="s">
-        <v>28</v>
-      </c>
-      <c r="R73" t="s">
-        <v>28</v>
-      </c>
-      <c r="S73" t="s">
-        <v>28</v>
-      </c>
-      <c r="T73" t="s">
-        <v>28</v>
-      </c>
-      <c r="U73" t="s">
-        <v>28</v>
-      </c>
-      <c r="V73" t="s">
-        <v>195</v>
-      </c>
-      <c r="W73" t="s">
-        <v>28</v>
-      </c>
-      <c r="X73" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y73" t="s">
+      <c r="D73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H73" s="4">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I73" s="4">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K73" s="4">
+        <v>2024</v>
+      </c>
+      <c r="L73" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N73" s="4">
+        <v>13</v>
+      </c>
+      <c r="O73" s="4">
+        <v>19</v>
+      </c>
+      <c r="P73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="R73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="S73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="T73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="U73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="V73" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="W73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="X73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y73" s="4" t="s">
         <v>194</v>
       </c>
     </row>
@@ -6292,10 +6292,10 @@
         <v>111</v>
       </c>
       <c r="B74" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="C74" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D74" t="s">
         <v>28</v>
@@ -6372,7 +6372,7 @@
         <v>134</v>
       </c>
       <c r="C75" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D75" t="s">
         <v>28</v>
@@ -6446,10 +6446,10 @@
         <v>111</v>
       </c>
       <c r="B76" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C76" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D76" t="s">
         <v>28</v>
@@ -6526,7 +6526,7 @@
         <v>137</v>
       </c>
       <c r="C77" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D77" t="s">
         <v>28</v>
@@ -6603,7 +6603,7 @@
         <v>137</v>
       </c>
       <c r="C78" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D78" t="s">
         <v>28</v>
@@ -6680,7 +6680,7 @@
         <v>137</v>
       </c>
       <c r="C79" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D79" t="s">
         <v>28</v>
@@ -6757,7 +6757,7 @@
         <v>137</v>
       </c>
       <c r="C80" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D80" t="s">
         <v>28</v>
@@ -6828,239 +6828,236 @@
     </row>
     <row r="81" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
+        <v>111</v>
+      </c>
+      <c r="B81" t="s">
+        <v>137</v>
+      </c>
+      <c r="C81" t="s">
+        <v>142</v>
+      </c>
+      <c r="D81" t="s">
+        <v>28</v>
+      </c>
+      <c r="E81" t="s">
+        <v>29</v>
+      </c>
+      <c r="F81" t="s">
+        <v>31</v>
+      </c>
+      <c r="G81" t="s">
+        <v>32</v>
+      </c>
+      <c r="H81">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I81">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J81" t="s">
+        <v>28</v>
+      </c>
+      <c r="K81">
+        <v>2024</v>
+      </c>
+      <c r="L81" t="s">
+        <v>33</v>
+      </c>
+      <c r="M81" t="s">
+        <v>28</v>
+      </c>
+      <c r="N81">
+        <v>13</v>
+      </c>
+      <c r="O81">
+        <v>19</v>
+      </c>
+      <c r="P81" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>28</v>
+      </c>
+      <c r="R81" t="s">
+        <v>28</v>
+      </c>
+      <c r="S81" t="s">
+        <v>28</v>
+      </c>
+      <c r="T81" t="s">
+        <v>28</v>
+      </c>
+      <c r="U81" t="s">
+        <v>28</v>
+      </c>
+      <c r="V81" t="s">
+        <v>195</v>
+      </c>
+      <c r="W81" t="s">
+        <v>28</v>
+      </c>
+      <c r="X81" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y81" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="82" spans="1:27" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>143</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B82" t="s">
         <v>143</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C82" t="s">
         <v>144</v>
       </c>
-      <c r="D81" t="s">
-        <v>28</v>
-      </c>
-      <c r="E81" t="s">
-        <v>29</v>
-      </c>
-      <c r="F81" t="s">
-        <v>31</v>
-      </c>
-      <c r="G81" t="s">
-        <v>32</v>
-      </c>
-      <c r="H81">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I81">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J81" t="s">
-        <v>28</v>
-      </c>
-      <c r="K81">
-        <v>2024</v>
-      </c>
-      <c r="L81" t="s">
-        <v>33</v>
-      </c>
-      <c r="M81" t="s">
-        <v>28</v>
-      </c>
-      <c r="N81">
-        <v>13</v>
-      </c>
-      <c r="O81">
-        <v>19</v>
-      </c>
-      <c r="P81" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q81" t="s">
-        <v>28</v>
-      </c>
-      <c r="R81" t="s">
-        <v>28</v>
-      </c>
-      <c r="S81" t="s">
-        <v>28</v>
-      </c>
-      <c r="T81" t="s">
-        <v>28</v>
-      </c>
-      <c r="U81" t="s">
-        <v>28</v>
-      </c>
-      <c r="V81" t="s">
-        <v>195</v>
-      </c>
-      <c r="W81" t="s">
-        <v>28</v>
-      </c>
-      <c r="X81" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y81" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="82" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="4" t="s">
+      <c r="D82" t="s">
+        <v>28</v>
+      </c>
+      <c r="E82" t="s">
+        <v>29</v>
+      </c>
+      <c r="F82" t="s">
+        <v>31</v>
+      </c>
+      <c r="G82" t="s">
+        <v>32</v>
+      </c>
+      <c r="H82">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I82">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J82" t="s">
+        <v>28</v>
+      </c>
+      <c r="K82">
+        <v>2024</v>
+      </c>
+      <c r="L82" t="s">
+        <v>33</v>
+      </c>
+      <c r="M82" t="s">
+        <v>28</v>
+      </c>
+      <c r="N82">
+        <v>13</v>
+      </c>
+      <c r="O82">
+        <v>19</v>
+      </c>
+      <c r="P82" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>28</v>
+      </c>
+      <c r="R82" t="s">
+        <v>28</v>
+      </c>
+      <c r="S82" t="s">
+        <v>28</v>
+      </c>
+      <c r="T82" t="s">
+        <v>28</v>
+      </c>
+      <c r="U82" t="s">
+        <v>28</v>
+      </c>
+      <c r="V82" t="s">
+        <v>195</v>
+      </c>
+      <c r="W82" t="s">
+        <v>28</v>
+      </c>
+      <c r="X82" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y82" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="83" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A83" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B82" s="4" t="s">
+      <c r="B83" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="C82" s="4" t="s">
+      <c r="C83" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="D82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="E82" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="F82" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="G82" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H82" s="4">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I82" s="4">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="K82" s="4">
-        <v>2024</v>
-      </c>
-      <c r="L82" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="N82" s="4">
-        <v>13</v>
-      </c>
-      <c r="O82" s="4">
-        <v>19</v>
-      </c>
-      <c r="P82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="R82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="S82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="T82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="U82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="V82" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="W82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="X82" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y82" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="AA82" s="4" t="s">
+      <c r="D83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G83" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H83" s="4">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I83" s="4">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="K83" s="4">
+        <v>2024</v>
+      </c>
+      <c r="L83" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="M83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="N83" s="4">
+        <v>13</v>
+      </c>
+      <c r="O83" s="4">
+        <v>19</v>
+      </c>
+      <c r="P83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="R83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="S83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="T83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="U83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="V83" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="W83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="X83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y83" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="AA83" s="4" t="s">
         <v>147</v>
-      </c>
-    </row>
-    <row r="83" spans="1:27" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
-        <v>143</v>
-      </c>
-      <c r="B83" t="s">
-        <v>143</v>
-      </c>
-      <c r="C83" t="s">
-        <v>146</v>
-      </c>
-      <c r="D83" t="s">
-        <v>28</v>
-      </c>
-      <c r="E83" t="s">
-        <v>29</v>
-      </c>
-      <c r="F83" t="s">
-        <v>31</v>
-      </c>
-      <c r="G83" t="s">
-        <v>32</v>
-      </c>
-      <c r="H83">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I83">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J83" t="s">
-        <v>28</v>
-      </c>
-      <c r="K83">
-        <v>2024</v>
-      </c>
-      <c r="L83" t="s">
-        <v>33</v>
-      </c>
-      <c r="M83" t="s">
-        <v>28</v>
-      </c>
-      <c r="N83">
-        <v>13</v>
-      </c>
-      <c r="O83">
-        <v>19</v>
-      </c>
-      <c r="P83" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q83" t="s">
-        <v>28</v>
-      </c>
-      <c r="R83" t="s">
-        <v>28</v>
-      </c>
-      <c r="S83" t="s">
-        <v>28</v>
-      </c>
-      <c r="T83" t="s">
-        <v>28</v>
-      </c>
-      <c r="U83" t="s">
-        <v>28</v>
-      </c>
-      <c r="V83" t="s">
-        <v>195</v>
-      </c>
-      <c r="W83" t="s">
-        <v>28</v>
-      </c>
-      <c r="X83" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y83" t="s">
-        <v>194</v>
-      </c>
-      <c r="AA83" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="84" spans="1:27" x14ac:dyDescent="0.35">
@@ -7068,10 +7065,10 @@
         <v>143</v>
       </c>
       <c r="B84" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="C84" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D84" t="s">
         <v>28</v>
@@ -7140,18 +7137,18 @@
         <v>194</v>
       </c>
       <c r="AA84" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="85" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="B85" t="s">
-        <v>28</v>
+        <v>152</v>
       </c>
       <c r="C85" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D85" t="s">
         <v>28</v>
@@ -7220,18 +7217,18 @@
         <v>194</v>
       </c>
       <c r="AA85" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="86" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B86" t="s">
         <v>28</v>
       </c>
       <c r="C86" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="D86" t="s">
         <v>28</v>
@@ -7300,7 +7297,7 @@
         <v>194</v>
       </c>
       <c r="AA86" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="87" spans="1:27" x14ac:dyDescent="0.35">
@@ -7311,7 +7308,7 @@
         <v>28</v>
       </c>
       <c r="C87" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D87" t="s">
         <v>28</v>
@@ -7378,17 +7375,20 @@
       </c>
       <c r="Y87" t="s">
         <v>194</v>
+      </c>
+      <c r="AA87" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="88" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B88" t="s">
         <v>28</v>
       </c>
       <c r="C88" t="s">
-        <v>100</v>
+        <v>158</v>
       </c>
       <c r="D88" t="s">
         <v>28</v>
@@ -7459,13 +7459,13 @@
     </row>
     <row r="89" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B89" t="s">
         <v>28</v>
       </c>
       <c r="C89" t="s">
-        <v>161</v>
+        <v>100</v>
       </c>
       <c r="D89" t="s">
         <v>28</v>
@@ -7536,13 +7536,13 @@
     </row>
     <row r="90" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B90" t="s">
-        <v>162</v>
+        <v>28</v>
       </c>
       <c r="C90" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D90" t="s">
         <v>28</v>
@@ -7619,7 +7619,7 @@
         <v>162</v>
       </c>
       <c r="C91" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D91" t="s">
         <v>28</v>
@@ -7696,7 +7696,7 @@
         <v>162</v>
       </c>
       <c r="C92" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D92" t="s">
         <v>28</v>
@@ -7767,13 +7767,13 @@
     </row>
     <row r="93" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B93" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="C93" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D93" t="s">
         <v>28</v>
@@ -7847,10 +7847,10 @@
         <v>166</v>
       </c>
       <c r="B94" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C94" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D94" t="s">
         <v>28</v>
@@ -7927,7 +7927,7 @@
         <v>166</v>
       </c>
       <c r="C95" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D95" t="s">
         <v>28</v>
@@ -7998,13 +7998,13 @@
     </row>
     <row r="96" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B96" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C96" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D96" t="s">
         <v>28</v>
@@ -8081,7 +8081,7 @@
         <v>172</v>
       </c>
       <c r="C97" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D97" t="s">
         <v>28</v>
@@ -8155,10 +8155,10 @@
         <v>171</v>
       </c>
       <c r="B98" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C98" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D98" t="s">
         <v>28</v>
@@ -8229,13 +8229,13 @@
     </row>
     <row r="99" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B99" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C99" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D99" t="s">
         <v>28</v>
@@ -8309,10 +8309,10 @@
         <v>177</v>
       </c>
       <c r="B100" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C100" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D100" t="s">
         <v>28</v>
@@ -8389,7 +8389,7 @@
         <v>180</v>
       </c>
       <c r="C101" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D101" t="s">
         <v>28</v>
@@ -8463,10 +8463,10 @@
         <v>177</v>
       </c>
       <c r="B102" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C102" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D102" t="s">
         <v>28</v>
@@ -8543,7 +8543,7 @@
         <v>177</v>
       </c>
       <c r="C103" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D103" t="s">
         <v>28</v>
@@ -8620,7 +8620,7 @@
         <v>177</v>
       </c>
       <c r="C104" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D104" t="s">
         <v>28</v>
@@ -8694,10 +8694,10 @@
         <v>177</v>
       </c>
       <c r="B105" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="C105" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D105" t="s">
         <v>28</v>
@@ -8774,7 +8774,7 @@
         <v>186</v>
       </c>
       <c r="C106" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D106" t="s">
         <v>28</v>
@@ -8845,13 +8845,13 @@
     </row>
     <row r="107" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B107" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C107" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D107" t="s">
         <v>28</v>
@@ -8928,7 +8928,7 @@
         <v>190</v>
       </c>
       <c r="C108" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D108" t="s">
         <v>28</v>
@@ -9005,77 +9005,154 @@
         <v>190</v>
       </c>
       <c r="C109" t="s">
+        <v>192</v>
+      </c>
+      <c r="D109" t="s">
+        <v>28</v>
+      </c>
+      <c r="E109" t="s">
+        <v>29</v>
+      </c>
+      <c r="F109" t="s">
+        <v>31</v>
+      </c>
+      <c r="G109" t="s">
+        <v>32</v>
+      </c>
+      <c r="H109">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I109">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J109" t="s">
+        <v>28</v>
+      </c>
+      <c r="K109">
+        <v>2024</v>
+      </c>
+      <c r="L109" t="s">
+        <v>33</v>
+      </c>
+      <c r="M109" t="s">
+        <v>28</v>
+      </c>
+      <c r="N109">
+        <v>13</v>
+      </c>
+      <c r="O109">
+        <v>19</v>
+      </c>
+      <c r="P109" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q109" t="s">
+        <v>28</v>
+      </c>
+      <c r="R109" t="s">
+        <v>28</v>
+      </c>
+      <c r="S109" t="s">
+        <v>28</v>
+      </c>
+      <c r="T109" t="s">
+        <v>28</v>
+      </c>
+      <c r="U109" t="s">
+        <v>28</v>
+      </c>
+      <c r="V109" t="s">
+        <v>195</v>
+      </c>
+      <c r="W109" t="s">
+        <v>28</v>
+      </c>
+      <c r="X109" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y109" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="110" spans="1:25" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>189</v>
+      </c>
+      <c r="B110" t="s">
+        <v>190</v>
+      </c>
+      <c r="C110" t="s">
         <v>193</v>
       </c>
-      <c r="D109" t="s">
-        <v>28</v>
-      </c>
-      <c r="E109" t="s">
-        <v>29</v>
-      </c>
-      <c r="F109" t="s">
-        <v>31</v>
-      </c>
-      <c r="G109" t="s">
-        <v>32</v>
-      </c>
-      <c r="H109">
-        <v>40.934753371594297</v>
-      </c>
-      <c r="I109">
-        <v>0.27523611725211999</v>
-      </c>
-      <c r="J109" t="s">
-        <v>28</v>
-      </c>
-      <c r="K109">
-        <v>2024</v>
-      </c>
-      <c r="L109" t="s">
-        <v>33</v>
-      </c>
-      <c r="M109" t="s">
-        <v>28</v>
-      </c>
-      <c r="N109">
-        <v>13</v>
-      </c>
-      <c r="O109">
-        <v>19</v>
-      </c>
-      <c r="P109" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q109" t="s">
-        <v>28</v>
-      </c>
-      <c r="R109" t="s">
-        <v>28</v>
-      </c>
-      <c r="S109" t="s">
-        <v>28</v>
-      </c>
-      <c r="T109" t="s">
-        <v>28</v>
-      </c>
-      <c r="U109" t="s">
-        <v>28</v>
-      </c>
-      <c r="V109" t="s">
-        <v>195</v>
-      </c>
-      <c r="W109" t="s">
-        <v>28</v>
-      </c>
-      <c r="X109" t="s">
-        <v>28</v>
-      </c>
-      <c r="Y109" t="s">
+      <c r="D110" t="s">
+        <v>28</v>
+      </c>
+      <c r="E110" t="s">
+        <v>29</v>
+      </c>
+      <c r="F110" t="s">
+        <v>31</v>
+      </c>
+      <c r="G110" t="s">
+        <v>32</v>
+      </c>
+      <c r="H110">
+        <v>40.934753371594297</v>
+      </c>
+      <c r="I110">
+        <v>0.27523611725211999</v>
+      </c>
+      <c r="J110" t="s">
+        <v>28</v>
+      </c>
+      <c r="K110">
+        <v>2024</v>
+      </c>
+      <c r="L110" t="s">
+        <v>33</v>
+      </c>
+      <c r="M110" t="s">
+        <v>28</v>
+      </c>
+      <c r="N110">
+        <v>13</v>
+      </c>
+      <c r="O110">
+        <v>19</v>
+      </c>
+      <c r="P110" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q110" t="s">
+        <v>28</v>
+      </c>
+      <c r="R110" t="s">
+        <v>28</v>
+      </c>
+      <c r="S110" t="s">
+        <v>28</v>
+      </c>
+      <c r="T110" t="s">
+        <v>28</v>
+      </c>
+      <c r="U110" t="s">
+        <v>28</v>
+      </c>
+      <c r="V110" t="s">
+        <v>195</v>
+      </c>
+      <c r="W110" t="s">
+        <v>28</v>
+      </c>
+      <c r="X110" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y110" t="s">
         <v>194</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA109"/>
+  <autoFilter ref="A1:AA110"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>